<commit_message>
add new outputs due to change of position of connector X6A
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_CarrierBoard/BOM/BOM_UZ_CarrierBoard_Rev05 - Mechanical Test.xlsx
+++ b/Project Outputs for UZ_CarrierBoard/BOM/BOM_UZ_CarrierBoard_Rev05 - Mechanical Test.xlsx
@@ -1,115 +1,85 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20412"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_carrier_board\Project Outputs for UZ_CarrierBoard\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\altium\uz_carrierboard\Project Outputs for UZ_CarrierBoard\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B93BE6-8B62-4B70-8557-8269B9D29CC8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{506CABB3-29A6-4344-9C9A-706EB1B35B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18400" windowHeight="9110" xr2:uid="{B743520C-1BF5-45C6-8CF8-52E1F9B9321F}"/>
+    <workbookView xWindow="-3135" yWindow="-11595" windowWidth="38700" windowHeight="15105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="BOM_UZ_CarrierBoard_Rev05 - Mec" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'BOM_UZ_CarrierBoard_Rev05 - Mec'!$1:$1</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
-  <si>
-    <t>Quantity</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Comment</t>
   </si>
   <si>
+    <t>HTEC8-150-01-L-DV-K</t>
+  </si>
+  <si>
     <t>Designator</t>
   </si>
   <si>
-    <t>MPN</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Description</t>
+    <t>X6A</t>
   </si>
   <si>
     <t>Footprint</t>
   </si>
   <si>
-    <t>Package</t>
-  </si>
-  <si>
-    <t>Voltage</t>
-  </si>
-  <si>
-    <t>Dielectric</t>
-  </si>
-  <si>
-    <t>Supplier 1</t>
-  </si>
-  <si>
-    <t>Supplier Part Number 1</t>
-  </si>
-  <si>
-    <t>Supplier 2</t>
-  </si>
-  <si>
-    <t>Supplier Part Number 2</t>
-  </si>
-  <si>
-    <t>Supplier 3</t>
-  </si>
-  <si>
-    <t>Supplier Part Number 3</t>
-  </si>
-  <si>
-    <t>HTEC8-150-01-L-DV-K</t>
-  </si>
-  <si>
-    <t>X6A</t>
-  </si>
-  <si>
-    <t>HTEC8-150-01-L-DV-K mating connector for card layout</t>
-  </si>
-  <si>
     <t>HTEC8-150-XX-X-DV</t>
   </si>
   <si>
-    <t>SAMTEC</t>
+    <t>LCSC Part Number</t>
   </si>
   <si>
     <t>C20365621</t>
-  </si>
-  <si>
-    <t>JLCPCB Part #</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -121,7 +91,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD3D3D3"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -136,29 +106,41 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -193,7 +175,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -205,7 +187,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -219,12 +201,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -252,31 +234,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -304,23 +269,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -463,126 +411,67 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D2B8047-BA9C-4970-8638-D3CDF0341B90}">
-  <dimension ref="A1:Q2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="10.1796875" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="18.1796875" customWidth="1"/>
-    <col min="5" max="5" width="20.36328125" customWidth="1"/>
-    <col min="6" max="6" width="13.26953125" customWidth="1"/>
-    <col min="7" max="9" width="12.36328125" customWidth="1"/>
-    <col min="10" max="10" width="9.453125" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" customWidth="1"/>
-    <col min="13" max="13" width="15.08984375" customWidth="1"/>
-    <col min="14" max="14" width="10.1796875" customWidth="1"/>
-    <col min="15" max="15" width="9" customWidth="1"/>
-    <col min="16" max="16" width="7.7265625" customWidth="1"/>
-    <col min="17" max="17" width="10.6328125" customWidth="1"/>
+    <col min="1" max="1" width="19.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>15</v>
-      </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
+    <row r="3" spans="1:4" ht="15.95" customHeight="1">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" ht="17.100000000000001" customHeight="1">
+      <c r="A4" s="2"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>